<commit_message>
Inclui P11074108 na NF 3611 com faturamento R$ 146,70 e custo R$ 92,68
O ribbon da FRANCAP não estava na planilha de agosto. Passa a entrar com
venda conferida R$ 146,70, custo R$ 92,68 e líquida R$ 54,02. A etiqueta
ETBOPP80185 da mesma nota permanece em R$ 5.166,90.

Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Faturamento Ago 2026.xlsx
+++ b/Faturamento Ago 2026.xlsx
@@ -1197,7 +1197,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42B2DAFE-0AE7-434A-A002-81D6B35C48F8}">
-  <dimension ref="A1:X134"/>
+  <dimension ref="A1:X135"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.54296875" bestFit="1" customWidth="1"/>
@@ -10046,6 +10046,58 @@
       <c r="R134" s="42"/>
       <c r="S134" s="43"/>
       <c r="T134" s="43"/>
+    </row>
+    <row r="135" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A135" s="11">
+        <v>3611</v>
+      </c>
+      <c r="B135" s="9">
+        <v>46245</v>
+      </c>
+      <c r="C135" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D135" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="E135" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="F135" s="11">
+        <v>30</v>
+      </c>
+      <c r="N135" s="24">
+        <v>2.64</v>
+      </c>
+      <c r="P135" s="16">
+        <v>79.2</v>
+      </c>
+      <c r="Q135" s="17">
+        <v>146.7</v>
+      </c>
+      <c r="R135" s="18">
+        <v>0</v>
+      </c>
+      <c r="S135" s="19">
+        <v>13.48</v>
+      </c>
+      <c r="T135" s="26">
+        <v>54.02</v>
+      </c>
+      <c r="U135" s="19">
+        <v>54.02</v>
+      </c>
+      <c r="V135" s="21">
+        <v>0.682070707070707</v>
+      </c>
+      <c r="W135" s="22">
+        <v>0</v>
+      </c>
+      <c r="X135" t="inlineStr">
+        <is>
+          <t>faturamento conferido R$ 146,70 · custo conferido R$ 92,68</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="U2:U62">

</xml_diff>

<commit_message>
Grava P11074108 da NF 3611 na planilha de agosto
A linha da FRANCAP fica na planilha com faturamento R$ 146,70, custo de
produto R$ 79,20 e imposto R$ 13,48 (custo total R$ 92,68).

Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Faturamento Ago 2026.xlsx
+++ b/Faturamento Ago 2026.xlsx
@@ -1197,7 +1197,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42B2DAFE-0AE7-434A-A002-81D6B35C48F8}">
-  <dimension ref="A1:X134"/>
+  <dimension ref="A1:X135"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.54296875" bestFit="1" customWidth="1"/>
@@ -10046,6 +10046,58 @@
       <c r="R134" s="42"/>
       <c r="S134" s="43"/>
       <c r="T134" s="43"/>
+    </row>
+    <row r="135" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="A135" s="11">
+        <v>3611</v>
+      </c>
+      <c r="B135" s="9">
+        <v>46245</v>
+      </c>
+      <c r="C135" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D135" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="E135" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="F135" s="11">
+        <v>30</v>
+      </c>
+      <c r="N135" s="24">
+        <v>2.64</v>
+      </c>
+      <c r="P135" s="16">
+        <v>79.2</v>
+      </c>
+      <c r="Q135" s="17">
+        <v>146.7</v>
+      </c>
+      <c r="R135" s="18">
+        <v>0</v>
+      </c>
+      <c r="S135" s="19">
+        <v>13.48</v>
+      </c>
+      <c r="T135" s="26">
+        <v>54.02</v>
+      </c>
+      <c r="U135" s="19">
+        <v>54.02</v>
+      </c>
+      <c r="V135" s="21">
+        <v>0.682070707070707</v>
+      </c>
+      <c r="W135" s="22">
+        <v>0</v>
+      </c>
+      <c r="X135" t="inlineStr">
+        <is>
+          <t>faturamento conferido R$ 146,70 · custo conferido R$ 92,68</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="U2:U62">

</xml_diff>